<commit_message>
Production file updates, m05 update in optomech
1) Added technical drawings to production folders and Adaptor folder.
2) Removed alignment pin holes from m05 in optomech.py as these were never real alignment pin holes.
3) Removed an outdated PD adaptor file from SAS Production Folder (PD_Adapter.step).
</commit_message>
<xml_diff>
--- a/Production/SASBoard/SAS_Board.xlsx
+++ b/Production/SASBoard/SAS_Board.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Github/PyOpticL_Rubidium_System/Production/SASBoard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josiahsinclair/Dropbox/2025-2032/SinclairLab/PyOpticL_Rubidium_System/Production/SASBoard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC48ED90-98C6-9145-BED5-BDED1D03E522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D90A34-C2D8-B743-A9E3-6A16F6CF2137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Adaptors</t>
   </si>
@@ -46,12 +46,6 @@
     <t>Surface_Adapter_rsp05_lip.step</t>
   </si>
   <si>
-    <t>Surface_Adapter_fiberport_lip.step</t>
-  </si>
-  <si>
-    <t>Cube_Mount.step</t>
-  </si>
-  <si>
     <t>M05</t>
   </si>
   <si>
@@ -98,6 +92,9 @@
   </si>
   <si>
     <t>SAS_Baseplate.step</t>
+  </si>
+  <si>
+    <t>Cube_Mount_Halfinch.step</t>
   </si>
 </sst>
 </file>
@@ -480,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504A0317-4413-EE44-9F8B-28AC1E65744B}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -488,7 +485,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -509,7 +506,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -517,7 +514,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -525,7 +522,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -533,63 +530,63 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12">
         <v>4</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -600,60 +597,52 @@
         <v>7</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>12</v>
+      <c r="A20" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A16" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
-    <hyperlink ref="A17" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
-    <hyperlink ref="A13" r:id="rId3" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
-    <hyperlink ref="A18" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
-    <hyperlink ref="A19" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
-    <hyperlink ref="A15" r:id="rId6" xr:uid="{6F72CF33-8356-4942-9395-81A746EF906E}"/>
-    <hyperlink ref="A21" r:id="rId7" xr:uid="{21E96D64-9EAA-B343-B30D-20CEC74ED8B8}"/>
-    <hyperlink ref="A22" r:id="rId8" xr:uid="{6D45723F-35A8-084B-9F84-679427F1593D}"/>
-    <hyperlink ref="A14" r:id="rId9" xr:uid="{504A2FB0-162D-DC40-91C8-F5121524BD11}"/>
+    <hyperlink ref="A15" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
+    <hyperlink ref="A16" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
+    <hyperlink ref="A12" r:id="rId3" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
+    <hyperlink ref="A17" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
+    <hyperlink ref="A18" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
+    <hyperlink ref="A14" r:id="rId6" xr:uid="{6F72CF33-8356-4942-9395-81A746EF906E}"/>
+    <hyperlink ref="A20" r:id="rId7" xr:uid="{21E96D64-9EAA-B343-B30D-20CEC74ED8B8}"/>
+    <hyperlink ref="A21" r:id="rId8" xr:uid="{6D45723F-35A8-084B-9F84-679427F1593D}"/>
+    <hyperlink ref="A13" r:id="rId9" xr:uid="{504A2FB0-162D-DC40-91C8-F5121524BD11}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>